<commit_message>
fix: repair liability persistence and access control
</commit_message>
<xml_diff>
--- a/backend/exports/责任不清报表_2026-06-11_1.xlsx
+++ b/backend/exports/责任不清报表_2026-06-11_1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>租约编号</t>
   </si>
@@ -44,6 +44,42 @@
   </si>
   <si>
     <t>营运人</t>
+  </si>
+  <si>
+    <t>OL2026063483</t>
+  </si>
+  <si>
+    <t>耐克 Nike</t>
+  </si>
+  <si>
+    <t>生效</t>
+  </si>
+  <si>
+    <t>LEASE_NO_RULE</t>
+  </si>
+  <si>
+    <t>未录入扣点(招商责任)</t>
+  </si>
+  <si>
+    <t>系统自动检测：提交租约时无扣点规则</t>
+  </si>
+  <si>
+    <t>张伟</t>
+  </si>
+  <si>
+    <t>2026-06-11 12:10:25</t>
+  </si>
+  <si>
+    <t>王强</t>
+  </si>
+  <si>
+    <t>OL2026069670</t>
+  </si>
+  <si>
+    <t>阿迪达斯 Adidas</t>
+  </si>
+  <si>
+    <t>待确认</t>
   </si>
 </sst>
 </file>
@@ -420,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -469,6 +505,73 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
fix: tighten dashboard access and rule supersede scope
</commit_message>
<xml_diff>
--- a/backend/exports/责任不清报表_2026-06-11_1.xlsx
+++ b/backend/exports/责任不清报表_2026-06-11_1.xlsx
@@ -46,7 +46,7 @@
     <t>营运人</t>
   </si>
   <si>
-    <t>OL2026063483</t>
+    <t>OL2026063754</t>
   </si>
   <si>
     <t>耐克 Nike</t>
@@ -67,13 +67,13 @@
     <t>张伟</t>
   </si>
   <si>
-    <t>2026-06-11 12:10:25</t>
+    <t>2026-06-11 12:21:28</t>
   </si>
   <si>
     <t>王强</t>
   </si>
   <si>
-    <t>OL2026069670</t>
+    <t>OL2026061236</t>
   </si>
   <si>
     <t>阿迪达斯 Adidas</t>

</xml_diff>

<commit_message>
feat: enrich supervisor liability progress filters
</commit_message>
<xml_diff>
--- a/backend/exports/责任不清报表_2026-06-11_1.xlsx
+++ b/backend/exports/责任不清报表_2026-06-11_1.xlsx
@@ -46,7 +46,7 @@
     <t>营运人</t>
   </si>
   <si>
-    <t>OL2026063754</t>
+    <t>OL2026065829</t>
   </si>
   <si>
     <t>耐克 Nike</t>
@@ -67,13 +67,13 @@
     <t>张伟</t>
   </si>
   <si>
-    <t>2026-06-11 12:21:28</t>
+    <t>2026-06-11 12:34:14</t>
   </si>
   <si>
     <t>王强</t>
   </si>
   <si>
-    <t>OL2026061236</t>
+    <t>OL2026067701</t>
   </si>
   <si>
     <t>阿迪达斯 Adidas</t>

</xml_diff>

<commit_message>
fix: align liability filters with latest deduction version
</commit_message>
<xml_diff>
--- a/backend/exports/责任不清报表_2026-06-11_1.xlsx
+++ b/backend/exports/责任不清报表_2026-06-11_1.xlsx
@@ -46,7 +46,7 @@
     <t>营运人</t>
   </si>
   <si>
-    <t>OL2026065829</t>
+    <t>OL2026064019</t>
   </si>
   <si>
     <t>耐克 Nike</t>
@@ -67,13 +67,13 @@
     <t>张伟</t>
   </si>
   <si>
-    <t>2026-06-11 12:34:14</t>
+    <t>2026-06-11 12:47:20</t>
   </si>
   <si>
     <t>王强</t>
   </si>
   <si>
-    <t>OL2026067701</t>
+    <t>OL2026065580</t>
   </si>
   <si>
     <t>阿迪达斯 Adidas</t>

</xml_diff>